<commit_message>
feat: torna pesquisas retomáveis e amplia cobertura do cache
</commit_message>
<xml_diff>
--- a/Planilha de Avaliação de Preços.xlsx
+++ b/Planilha de Avaliação de Preços.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PNCPKing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFCAC71-366F-4483-8D02-EB46819725C3}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFEB252-5469-401B-905F-0F8F77E10EF6}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
   <si>
     <t>PLANILHA DE AVALIAÇÃO DE PREÇOS</t>
   </si>
@@ -109,6 +109,12 @@
   <si>
     <t>{{ preco.empresa_nome }} {{da cidade de, Estado de}}</t>
   </si>
+  <si>
+    <t>Responsável pela cotação:</t>
+  </si>
+  <si>
+    <t>NOME DO USUÁRIO                                                                                                                               AGENTE DE ADMINISTRAÇÃO</t>
+  </si>
 </sst>
 </file>
 
@@ -117,7 +123,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.0000;\-&quot;R$&quot;\ #,##0.0000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -173,8 +179,32 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,8 +223,14 @@
         <bgColor rgb="FFD0CECE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -458,11 +494,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -575,6 +657,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1868,7 +1968,7 @@
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
     </row>
-    <row r="24" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:27" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1897,36 +1997,40 @@
       <c r="Z24" s="2"/>
       <c r="AA24" s="2"/>
     </row>
-    <row r="25" spans="1:27" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="2"/>
-      <c r="W25" s="2"/>
-      <c r="X25" s="2"/>
-      <c r="Y25" s="2"/>
-      <c r="Z25" s="2"/>
+    <row r="25" spans="1:27" ht="77.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="44"/>
+      <c r="B25" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="46"/>
+      <c r="K25" s="46"/>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="46"/>
+      <c r="Q25" s="46"/>
+      <c r="R25" s="46"/>
+      <c r="S25" s="46"/>
+      <c r="T25" s="46"/>
+      <c r="U25" s="46"/>
+      <c r="V25" s="46"/>
+      <c r="W25" s="46"/>
+      <c r="X25" s="46"/>
+      <c r="Y25" s="46"/>
+      <c r="Z25" s="46"/>
       <c r="AA25" s="2"/>
     </row>
-    <row r="26" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:27" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -27795,10 +27899,11 @@
       <c r="AA917" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C25:H25"/>
   </mergeCells>
   <conditionalFormatting sqref="H3 H6:H24">
     <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="EXCESSIVO">
@@ -27821,7 +27926,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>